<commit_message>
Atualiza apontamento servicos e arquivos correlatos
</commit_message>
<xml_diff>
--- a/tmp/04 ATESTE BT PF NEG TEST.xlsx
+++ b/tmp/04 ATESTE BT PF NEG TEST.xlsx
@@ -435,6 +435,18 @@
       <c r="T6">
         <v>-14</v>
       </c>
+      <c r="U6">
+        <v>4</v>
+      </c>
+      <c r="V6">
+        <v>-3</v>
+      </c>
+      <c r="W6">
+        <v>2</v>
+      </c>
+      <c r="X6">
+        <v>-1</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="str">
@@ -461,6 +473,18 @@
       <c r="T7">
         <v>-24</v>
       </c>
+      <c r="U7">
+        <v>8</v>
+      </c>
+      <c r="V7">
+        <v>-7</v>
+      </c>
+      <c r="W7">
+        <v>6</v>
+      </c>
+      <c r="X7">
+        <v>-5</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="str">
@@ -487,6 +511,18 @@
       <c r="T8">
         <v>-34</v>
       </c>
+      <c r="U8">
+        <v>12</v>
+      </c>
+      <c r="V8">
+        <v>-11</v>
+      </c>
+      <c r="W8">
+        <v>10</v>
+      </c>
+      <c r="X8">
+        <v>-9</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="str">
@@ -513,6 +549,18 @@
       <c r="T9">
         <v>-44</v>
       </c>
+      <c r="U9">
+        <v>16</v>
+      </c>
+      <c r="V9">
+        <v>-15</v>
+      </c>
+      <c r="W9">
+        <v>14</v>
+      </c>
+      <c r="X9">
+        <v>-13</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="str">
@@ -538,6 +586,18 @@
       </c>
       <c r="T10">
         <v>-54</v>
+      </c>
+      <c r="U10">
+        <v>20</v>
+      </c>
+      <c r="V10">
+        <v>-19</v>
+      </c>
+      <c r="W10">
+        <v>18</v>
+      </c>
+      <c r="X10">
+        <v>-17</v>
       </c>
     </row>
   </sheetData>
@@ -561,6 +621,12 @@
       <c r="M6">
         <v>-16</v>
       </c>
+      <c r="N6">
+        <v>6</v>
+      </c>
+      <c r="O6">
+        <v>-5</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="str">
@@ -572,6 +638,12 @@
       <c r="M7">
         <v>-26</v>
       </c>
+      <c r="N7">
+        <v>10</v>
+      </c>
+      <c r="O7">
+        <v>-9</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="str">
@@ -583,6 +655,12 @@
       <c r="M8">
         <v>-36</v>
       </c>
+      <c r="N8">
+        <v>14</v>
+      </c>
+      <c r="O8">
+        <v>-13</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="str">
@@ -594,6 +672,12 @@
       <c r="M9">
         <v>-46</v>
       </c>
+      <c r="N9">
+        <v>18</v>
+      </c>
+      <c r="O9">
+        <v>-17</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="str">
@@ -604,6 +688,12 @@
       </c>
       <c r="M10">
         <v>-56</v>
+      </c>
+      <c r="N10">
+        <v>22</v>
+      </c>
+      <c r="O10">
+        <v>-21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>